<commit_message>
feat: agregar vendedor FERNANDO, forma de pago NO PAGO en rojo y resumenes de excel
</commit_message>
<xml_diff>
--- a/test_export_real.xlsx
+++ b/test_export_real.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="27">
   <si>
     <t>INFORME DE VENTAS DEL DÍA</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>ANDRES Jr.</t>
+  </si>
+  <si>
+    <t>LOCAL</t>
   </si>
   <si>
     <t>🔍 BUSCADOR INTELIGENTE DE VENTAS — Comedor Donde Flory</t>
@@ -571,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -780,6 +783,32 @@
       </c>
       <c r="G21" s="11">
         <f>SUMIFS(E3:E5, G3:G5, "ANDRES Jr.", F3:F5, "TARJETA")</f>
+      </c>
+    </row>
+    <row r="23" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D23" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D24" s="10"/>
+      <c r="E24" s="11">
+        <f>SUMIFS(E3:E5, G3:G5, "LOCAL", F3:F5, "EFECTIVO")</f>
+      </c>
+      <c r="F24" s="11">
+        <f>SUMIFS(E3:E5, G3:G5, "LOCAL", F3:F5, "TRANSFERENCIA")</f>
+      </c>
+      <c r="G24" s="11">
+        <f>SUMIFS(E3:E5, G3:G5, "LOCAL", F3:F5, "TARJETA")</f>
       </c>
     </row>
   </sheetData>
@@ -807,7 +836,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -818,7 +847,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -829,10 +858,10 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="3:5" x14ac:dyDescent="0.25">
@@ -848,7 +877,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>4</v>
@@ -898,7 +927,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="C4">
-      <formula1>"FREDY,JAIME,VIEJO,ANDRES Jr.,OTROS"</formula1>
+      <formula1>"FREDY,JAIME,VIEJO,ANDRES Jr.,LOCAL,OTROS"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E4">
       <formula1>"EFECTIVO,TRANSFERENCIA,TARJETA"</formula1>

</xml_diff>